<commit_message>
finished up battle relics
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configurations/NewCards.xlsx
+++ b/Assets/StreamingAssets/Configurations/NewCards.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\VTuberSim\Assets\StreamingAssets\Configurations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{896509AF-F5C6-4E31-9F13-A26265473CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9618729-529B-4113-9140-C2D3C826719B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="5" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25490" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cards" sheetId="1" r:id="rId1"/>
@@ -21,9 +21,9 @@
     <sheet name="CardConditions" sheetId="6" r:id="rId6"/>
     <sheet name="StreamEvents" sheetId="8" r:id="rId7"/>
     <sheet name="DialogueEvents" sheetId="7" r:id="rId8"/>
-    <sheet name="PhaseEndingConditions" sheetId="10" r:id="rId9"/>
-    <sheet name="Relics" sheetId="11" r:id="rId10"/>
-    <sheet name="RaisingRelicConditions" sheetId="13" r:id="rId11"/>
+    <sheet name="RaisingRelicConditions" sheetId="13" r:id="rId9"/>
+    <sheet name="PhaseEndingConditions" sheetId="10" r:id="rId10"/>
+    <sheet name="Relics" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cards!$A$1:$AE$61</definedName>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="394">
   <si>
     <t>ID</t>
   </si>
@@ -1162,12 +1162,6 @@
     <t>Layer</t>
   </si>
   <si>
-    <t>VBattleRelicConfiguration</t>
-  </si>
-  <si>
-    <t>OnTurnBegin</t>
-  </si>
-  <si>
     <t>VCardOperationRelicCondition</t>
   </si>
   <si>
@@ -1214,6 +1208,24 @@
   </si>
   <si>
     <t>获得神采100%的参数，下一回合抽一张卡牌</t>
+  </si>
+  <si>
+    <t>AddRelic0</t>
+  </si>
+  <si>
+    <t>VRaisingAddRelicEffect</t>
+  </si>
+  <si>
+    <t>VBattleRelic</t>
+  </si>
+  <si>
+    <t>MyRelic</t>
+  </si>
+  <si>
+    <t>VCardTypeUsedCountCondition</t>
+  </si>
+  <si>
+    <t>OnCardUsed</t>
   </si>
 </sst>
 </file>
@@ -1626,7 +1638,7 @@
   <cols>
     <col min="1" max="1" width="3.42578125" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="3" max="3" width="37.7109375" customWidth="1"/>
     <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="13.42578125" customWidth="1"/>
     <col min="6" max="6" width="10.5703125" customWidth="1"/>
@@ -1857,7 +1869,7 @@
         <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D4" t="s">
         <v>32</v>
@@ -1968,10 +1980,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="C6" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D6" t="s">
         <v>43</v>
@@ -3561,7 +3573,7 @@
         <v>100</v>
       </c>
       <c r="C33" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D33" t="s">
         <v>43</v>
@@ -3634,9 +3646,6 @@
       <c r="K34">
         <v>0</v>
       </c>
-      <c r="L34" s="9">
-        <v>0</v>
-      </c>
       <c r="M34" s="7">
         <v>15</v>
       </c>
@@ -3655,10 +3664,10 @@
         <v>36</v>
       </c>
       <c r="B35" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C35" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D35" t="s">
         <v>61</v>
@@ -4997,10 +5006,10 @@
         <v>59</v>
       </c>
       <c r="B58" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C58" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D58" t="s">
         <v>32</v>
@@ -5032,10 +5041,10 @@
         <v>60</v>
       </c>
       <c r="B59" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C59" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D59" t="s">
         <v>61</v>
@@ -5076,10 +5085,10 @@
         <v>61</v>
       </c>
       <c r="B60" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C60" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D60" t="s">
         <v>43</v>
@@ -5111,10 +5120,10 @@
         <v>62</v>
       </c>
       <c r="B61" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C61" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D61" t="s">
         <v>61</v>
@@ -5156,6 +5165,104 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6620075D-DE02-4F16-B523-AE1F397F6AC8}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.42578125" customWidth="1"/>
+    <col min="3" max="3" width="22.85546875" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="C2">
+        <v>36</v>
+      </c>
+      <c r="D2" t="s">
+        <v>349</v>
+      </c>
+      <c r="E2" t="s">
+        <v>287</v>
+      </c>
+      <c r="F2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>12</v>
+      </c>
+      <c r="C3">
+        <v>36</v>
+      </c>
+      <c r="D3" t="s">
+        <v>349</v>
+      </c>
+      <c r="E3" t="s">
+        <v>287</v>
+      </c>
+      <c r="F3">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
+      <c r="C4">
+        <v>36</v>
+      </c>
+      <c r="D4" t="s">
+        <v>351</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAFA4640-CFCE-465A-87A0-93766D6720A8}">
   <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -5164,7 +5271,7 @@
     <col min="3" max="3" width="18.85546875" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" customWidth="1"/>
     <col min="7" max="7" width="11.85546875" customWidth="1"/>
     <col min="8" max="8" width="10.28515625" customWidth="1"/>
     <col min="9" max="9" width="13.140625" customWidth="1"/>
@@ -5234,85 +5341,32 @@
       <c r="A2">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>1</v>
+      <c r="B2" t="s">
+        <v>391</v>
       </c>
       <c r="C2">
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
       <c r="E2">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F9A170A-FBD6-48B2-AAE0-2B7F0755C3F2}">
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="12.140625" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
-    <col min="3" max="3" width="15.42578125" customWidth="1"/>
-    <col min="4" max="4" width="28.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>368</v>
-      </c>
-      <c r="F1" t="s">
-        <v>369</v>
-      </c>
-      <c r="G1" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>374</v>
-      </c>
-      <c r="E2" t="s">
-        <v>375</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>38</v>
+        <v>393</v>
+      </c>
+      <c r="G2">
+        <v>9</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -7222,12 +7276,12 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.85546875" customWidth="1"/>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.7109375" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" customWidth="1"/>
     <col min="5" max="5" width="16.140625" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
@@ -7431,15 +7485,35 @@
         <v>50</v>
       </c>
     </row>
+    <row r="11" spans="1:7">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>12313</v>
+      </c>
+      <c r="C11" t="s">
+        <v>392</v>
+      </c>
+      <c r="D11" t="s">
+        <v>273</v>
+      </c>
+      <c r="E11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="31.42578125" customWidth="1"/>
@@ -7691,7 +7765,25 @@
         <v>2</v>
       </c>
     </row>
+    <row r="15" spans="1:6">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>388</v>
+      </c>
+      <c r="C15" t="s">
+        <v>388</v>
+      </c>
+      <c r="D15" t="s">
+        <v>389</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -8662,19 +8754,19 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6620075D-DE02-4F16-B523-AE1F397F6AC8}">
-  <dimension ref="A1:F4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F9A170A-FBD6-48B2-AAE0-2B7F0755C3F2}">
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="22.85546875" customWidth="1"/>
-    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.42578125" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8688,73 +8780,40 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>268</v>
+        <v>368</v>
       </c>
       <c r="F1" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>369</v>
+      </c>
+      <c r="G1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>349</v>
+        <v>372</v>
       </c>
       <c r="E2" t="s">
-        <v>287</v>
-      </c>
-      <c r="F2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>12</v>
-      </c>
-      <c r="C3">
-        <v>36</v>
-      </c>
-      <c r="D3" t="s">
-        <v>349</v>
-      </c>
-      <c r="E3" t="s">
-        <v>287</v>
-      </c>
-      <c r="F3">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4">
-        <v>12</v>
-      </c>
-      <c r="C4">
-        <v>36</v>
-      </c>
-      <c r="D4" t="s">
-        <v>351</v>
-      </c>
-      <c r="E4">
-        <v>5</v>
-      </c>
-      <c r="F4" t="s">
-        <v>319</v>
+        <v>373</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>